<commit_message>
refactor: switch all units to US (in / lb / ft / cft) + add per-load utilization %
- Master data: width/depth/height in inches, weight in lb, volume in cft
- Truck data: length/width/height in inches, payload in lb, cargo in cft
- best_packer: door track loss 10 in (was 250 mm), all internal math in inches
- Excel Calculator: direct VLOOKUP in/lb (no conversion factors)
  + per-load Length/Volume/Weight utilization % with green/orange/gray bands
- Tests: updated to US units, AABB overlap check now uses 0.05 in tolerance
- 13/13 packer tests passing
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Master" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loads" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Truck_Master" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Model_Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Truck_Master" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Loads" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,64 +431,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model_code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>width_mm</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>depth_mm</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>height_mm</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>weight_kg</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>width_in</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>depth_in</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>height_in</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>weight_lb</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>this_side_up</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>stackable</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>load_bear_kg</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>load_bear_lb</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>fragile</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>volume_cbm</t>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>volume_cft</t>
         </is>
       </c>
     </row>
@@ -492,16 +504,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>940</v>
+        <v>37.01</v>
       </c>
       <c r="D2" t="n">
-        <v>900</v>
+        <v>35.43</v>
       </c>
       <c r="E2" t="n">
-        <v>1850</v>
+        <v>72.83</v>
       </c>
       <c r="F2" t="n">
-        <v>155</v>
+        <v>341.7</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -521,7 +533,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>1.5651</v>
+        <v>55.27</v>
       </c>
     </row>
     <row r="3">
@@ -536,16 +548,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>860</v>
+        <v>33.86</v>
       </c>
       <c r="D3" t="n">
-        <v>820</v>
+        <v>32.28</v>
       </c>
       <c r="E3" t="n">
-        <v>1810</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>135</v>
+        <v>297.6</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -565,7 +577,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>1.2764</v>
+        <v>45.08</v>
       </c>
     </row>
     <row r="4">
@@ -580,16 +592,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>920</v>
+        <v>36.22</v>
       </c>
       <c r="D4" t="n">
-        <v>770</v>
+        <v>30.31</v>
       </c>
       <c r="E4" t="n">
-        <v>1840</v>
+        <v>72.44</v>
       </c>
       <c r="F4" t="n">
-        <v>140</v>
+        <v>308.6</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -609,7 +621,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1.3035</v>
+        <v>46.03</v>
       </c>
     </row>
     <row r="5">
@@ -624,16 +636,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>960</v>
+        <v>37.8</v>
       </c>
       <c r="D5" t="n">
-        <v>880</v>
+        <v>34.65</v>
       </c>
       <c r="E5" t="n">
-        <v>1870</v>
+        <v>73.62</v>
       </c>
       <c r="F5" t="n">
-        <v>160</v>
+        <v>352.7</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -653,7 +665,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>1.5798</v>
+        <v>55.79</v>
       </c>
     </row>
     <row r="6">
@@ -668,16 +680,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>850</v>
+        <v>33.46</v>
       </c>
       <c r="D6" t="n">
-        <v>780</v>
+        <v>30.71</v>
       </c>
       <c r="E6" t="n">
-        <v>1800</v>
+        <v>70.87</v>
       </c>
       <c r="F6" t="n">
-        <v>125</v>
+        <v>275.6</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -697,7 +709,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>1.1934</v>
+        <v>42.14</v>
       </c>
     </row>
     <row r="7">
@@ -712,16 +724,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>910</v>
+        <v>35.83</v>
       </c>
       <c r="D7" t="n">
-        <v>820</v>
+        <v>32.28</v>
       </c>
       <c r="E7" t="n">
-        <v>1810</v>
+        <v>71.26000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>130</v>
+        <v>286.6</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -741,7 +753,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>1.3506</v>
+        <v>47.7</v>
       </c>
     </row>
     <row r="8">
@@ -756,16 +768,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>745</v>
+        <v>29.33</v>
       </c>
       <c r="D8" t="n">
-        <v>830</v>
+        <v>32.68</v>
       </c>
       <c r="E8" t="n">
-        <v>1050</v>
+        <v>41.34</v>
       </c>
       <c r="F8" t="n">
-        <v>95</v>
+        <v>209.4</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -774,7 +786,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>95</v>
+        <v>209.4</v>
       </c>
       <c r="J8" t="b">
         <v>0</v>
@@ -785,7 +797,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.6493</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="9">
@@ -800,16 +812,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>745</v>
+        <v>29.33</v>
       </c>
       <c r="D9" t="n">
-        <v>830</v>
+        <v>32.68</v>
       </c>
       <c r="E9" t="n">
-        <v>1050</v>
+        <v>41.34</v>
       </c>
       <c r="F9" t="n">
-        <v>75</v>
+        <v>165.3</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -818,7 +830,7 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>95</v>
+        <v>209.4</v>
       </c>
       <c r="J9" t="b">
         <v>0</v>
@@ -829,7 +841,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.6493</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="10">
@@ -844,16 +856,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>745</v>
+        <v>29.33</v>
       </c>
       <c r="D10" t="n">
-        <v>830</v>
+        <v>32.68</v>
       </c>
       <c r="E10" t="n">
-        <v>1050</v>
+        <v>41.34</v>
       </c>
       <c r="F10" t="n">
-        <v>80</v>
+        <v>176.4</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -862,7 +874,7 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>95</v>
+        <v>209.4</v>
       </c>
       <c r="J10" t="b">
         <v>0</v>
@@ -873,7 +885,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.6493</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="11">
@@ -888,16 +900,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>720</v>
+        <v>28.35</v>
       </c>
       <c r="D11" t="n">
-        <v>770</v>
+        <v>30.31</v>
       </c>
       <c r="E11" t="n">
-        <v>1170</v>
+        <v>46.06</v>
       </c>
       <c r="F11" t="n">
-        <v>70</v>
+        <v>154.3</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -917,7 +929,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0.6486</v>
+        <v>22.91</v>
       </c>
     </row>
     <row r="12">
@@ -932,16 +944,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>670</v>
+        <v>26.38</v>
       </c>
       <c r="D12" t="n">
-        <v>730</v>
+        <v>28.74</v>
       </c>
       <c r="E12" t="n">
-        <v>920</v>
+        <v>36.22</v>
       </c>
       <c r="F12" t="n">
-        <v>55</v>
+        <v>121.3</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
@@ -961,7 +973,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>0.45</v>
+        <v>15.89</v>
       </c>
     </row>
     <row r="13">
@@ -976,16 +988,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>830</v>
+        <v>32.68</v>
       </c>
       <c r="D13" t="n">
-        <v>790</v>
+        <v>31.1</v>
       </c>
       <c r="E13" t="n">
-        <v>1230</v>
+        <v>48.43</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>220.5</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
@@ -1005,7 +1017,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0.8065</v>
+        <v>28.48</v>
       </c>
     </row>
     <row r="14">
@@ -1020,16 +1032,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>830</v>
+        <v>32.68</v>
       </c>
       <c r="D14" t="n">
-        <v>790</v>
+        <v>31.1</v>
       </c>
       <c r="E14" t="n">
-        <v>1230</v>
+        <v>48.43</v>
       </c>
       <c r="F14" t="n">
-        <v>90</v>
+        <v>198.4</v>
       </c>
       <c r="G14" t="b">
         <v>1</v>
@@ -1049,7 +1061,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>0.8065</v>
+        <v>28.48</v>
       </c>
     </row>
     <row r="15">
@@ -1064,16 +1076,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>820</v>
+        <v>32.28</v>
       </c>
       <c r="D15" t="n">
-        <v>720</v>
+        <v>28.35</v>
       </c>
       <c r="E15" t="n">
-        <v>890</v>
+        <v>35.04</v>
       </c>
       <c r="F15" t="n">
-        <v>85</v>
+        <v>187.4</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
@@ -1093,7 +1105,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>0.5255</v>
+        <v>18.56</v>
       </c>
     </row>
     <row r="16">
@@ -1108,16 +1120,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>820</v>
+        <v>32.28</v>
       </c>
       <c r="D16" t="n">
-        <v>520</v>
+        <v>20.47</v>
       </c>
       <c r="E16" t="n">
-        <v>500</v>
+        <v>19.69</v>
       </c>
       <c r="F16" t="n">
-        <v>28</v>
+        <v>61.7</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
@@ -1126,7 +1138,7 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>30</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="J16" t="b">
         <v>0</v>
@@ -1137,7 +1149,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>0.2132</v>
+        <v>7.53</v>
       </c>
     </row>
     <row r="17">
@@ -1152,16 +1164,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>620</v>
+        <v>24.41</v>
       </c>
       <c r="D17" t="n">
-        <v>510</v>
+        <v>20.08</v>
       </c>
       <c r="E17" t="n">
-        <v>410</v>
+        <v>16.14</v>
       </c>
       <c r="F17" t="n">
-        <v>18</v>
+        <v>39.7</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
@@ -1170,7 +1182,7 @@
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>20</v>
+        <v>44.1</v>
       </c>
       <c r="J17" t="b">
         <v>0</v>
@@ -1181,7 +1193,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>0.1296</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="18">
@@ -1196,16 +1208,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1665</v>
+        <v>65.55</v>
       </c>
       <c r="D18" t="n">
-        <v>205</v>
+        <v>8.07</v>
       </c>
       <c r="E18" t="n">
-        <v>975</v>
+        <v>38.39</v>
       </c>
       <c r="F18" t="n">
-        <v>24</v>
+        <v>52.9</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
@@ -1214,7 +1226,7 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J18" t="b">
         <v>1</v>
@@ -1225,7 +1237,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0.3328</v>
+        <v>11.75</v>
       </c>
     </row>
     <row r="19">
@@ -1240,16 +1252,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1900</v>
+        <v>74.8</v>
       </c>
       <c r="D19" t="n">
-        <v>285</v>
+        <v>11.22</v>
       </c>
       <c r="E19" t="n">
-        <v>1135</v>
+        <v>44.69</v>
       </c>
       <c r="F19" t="n">
-        <v>50</v>
+        <v>110.2</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
@@ -1258,7 +1270,7 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J19" t="b">
         <v>1</v>
@@ -1269,7 +1281,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>0.6146</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="20">
@@ -1284,16 +1296,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2040</v>
+        <v>80.31</v>
       </c>
       <c r="D20" t="n">
-        <v>305</v>
+        <v>12.01</v>
       </c>
       <c r="E20" t="n">
-        <v>1230</v>
+        <v>48.43</v>
       </c>
       <c r="F20" t="n">
-        <v>62</v>
+        <v>136.7</v>
       </c>
       <c r="G20" t="b">
         <v>1</v>
@@ -1313,7 +1325,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>0.7653</v>
+        <v>27.03</v>
       </c>
     </row>
     <row r="21">
@@ -1328,16 +1340,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1430</v>
+        <v>56.3</v>
       </c>
       <c r="D21" t="n">
-        <v>195</v>
+        <v>7.68</v>
       </c>
       <c r="E21" t="n">
-        <v>855</v>
+        <v>33.66</v>
       </c>
       <c r="F21" t="n">
-        <v>18</v>
+        <v>39.7</v>
       </c>
       <c r="G21" t="b">
         <v>1</v>
@@ -1346,7 +1358,7 @@
         <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J21" t="b">
         <v>1</v>
@@ -1357,7 +1369,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>0.2384</v>
+        <v>8.42</v>
       </c>
     </row>
     <row r="22">
@@ -1372,16 +1384,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1675</v>
+        <v>65.94</v>
       </c>
       <c r="D22" t="n">
-        <v>225</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>985</v>
+        <v>38.78</v>
       </c>
       <c r="F22" t="n">
-        <v>28</v>
+        <v>61.7</v>
       </c>
       <c r="G22" t="b">
         <v>1</v>
@@ -1390,7 +1402,7 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J22" t="b">
         <v>1</v>
@@ -1401,7 +1413,7 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>0.3712</v>
+        <v>13.11</v>
       </c>
     </row>
     <row r="23">
@@ -1416,16 +1428,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1820</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="D23" t="n">
-        <v>255</v>
+        <v>10.04</v>
       </c>
       <c r="E23" t="n">
-        <v>1110</v>
+        <v>43.7</v>
       </c>
       <c r="F23" t="n">
-        <v>42</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G23" t="b">
         <v>1</v>
@@ -1434,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J23" t="b">
         <v>1</v>
@@ -1445,7 +1457,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>0.5152</v>
+        <v>18.19</v>
       </c>
     </row>
     <row r="24">
@@ -1460,16 +1472,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1240</v>
+        <v>48.82</v>
       </c>
       <c r="D24" t="n">
-        <v>175</v>
+        <v>6.89</v>
       </c>
       <c r="E24" t="n">
-        <v>790</v>
+        <v>31.1</v>
       </c>
       <c r="F24" t="n">
-        <v>14</v>
+        <v>30.9</v>
       </c>
       <c r="G24" t="b">
         <v>1</v>
@@ -1478,7 +1490,7 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J24" t="b">
         <v>1</v>
@@ -1489,7 +1501,7 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>0.1714</v>
+        <v>6.05</v>
       </c>
     </row>
     <row r="25">
@@ -1504,16 +1516,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1100</v>
+        <v>43.31</v>
       </c>
       <c r="D25" t="n">
-        <v>165</v>
+        <v>6.5</v>
       </c>
       <c r="E25" t="n">
-        <v>705</v>
+        <v>27.76</v>
       </c>
       <c r="F25" t="n">
-        <v>11</v>
+        <v>24.3</v>
       </c>
       <c r="G25" t="b">
         <v>1</v>
@@ -1522,7 +1534,7 @@
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>15</v>
+        <v>33.1</v>
       </c>
       <c r="J25" t="b">
         <v>1</v>
@@ -1533,7 +1545,7 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>0.128</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="26">
@@ -1548,16 +1560,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>770</v>
+        <v>30.31</v>
       </c>
       <c r="D26" t="n">
-        <v>200</v>
+        <v>7.87</v>
       </c>
       <c r="E26" t="n">
-        <v>495</v>
+        <v>19.49</v>
       </c>
       <c r="F26" t="n">
-        <v>9</v>
+        <v>19.8</v>
       </c>
       <c r="G26" t="b">
         <v>1</v>
@@ -1566,7 +1578,7 @@
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>12</v>
+        <v>26.5</v>
       </c>
       <c r="J26" t="b">
         <v>1</v>
@@ -1577,7 +1589,7 @@
         </is>
       </c>
       <c r="L26" t="n">
-        <v>0.0762</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="27">
@@ -1592,16 +1604,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>860</v>
+        <v>33.86</v>
       </c>
       <c r="D27" t="n">
-        <v>220</v>
+        <v>8.66</v>
       </c>
       <c r="E27" t="n">
-        <v>560</v>
+        <v>22.05</v>
       </c>
       <c r="F27" t="n">
-        <v>11</v>
+        <v>24.3</v>
       </c>
       <c r="G27" t="b">
         <v>1</v>
@@ -1610,7 +1622,7 @@
         <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>12</v>
+        <v>26.5</v>
       </c>
       <c r="J27" t="b">
         <v>1</v>
@@ -1621,7 +1633,7 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>0.106</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="28">
@@ -1636,16 +1648,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>880</v>
+        <v>34.65</v>
       </c>
       <c r="D28" t="n">
-        <v>230</v>
+        <v>9.06</v>
       </c>
       <c r="E28" t="n">
-        <v>580</v>
+        <v>22.83</v>
       </c>
       <c r="F28" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
       <c r="G28" t="b">
         <v>1</v>
@@ -1654,7 +1666,7 @@
         <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>12</v>
+        <v>26.5</v>
       </c>
       <c r="J28" t="b">
         <v>1</v>
@@ -1665,7 +1677,7 @@
         </is>
       </c>
       <c r="L28" t="n">
-        <v>0.1174</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="29">
@@ -1680,16 +1692,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>770</v>
+        <v>30.31</v>
       </c>
       <c r="D29" t="n">
-        <v>200</v>
+        <v>7.87</v>
       </c>
       <c r="E29" t="n">
-        <v>495</v>
+        <v>19.49</v>
       </c>
       <c r="F29" t="n">
-        <v>9</v>
+        <v>19.8</v>
       </c>
       <c r="G29" t="b">
         <v>1</v>
@@ -1698,7 +1710,7 @@
         <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>12</v>
+        <v>26.5</v>
       </c>
       <c r="J29" t="b">
         <v>1</v>
@@ -1709,7 +1721,7 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>0.0762</v>
+        <v>2.69</v>
       </c>
     </row>
   </sheetData>
@@ -1723,549 +1735,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>load_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>model_code</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>destination</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>pickup_date</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>truck_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>length_in</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>width_in</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>height_in</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>max_payload_lb</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>cargo_volume_cft</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L001</t>
+          <t>26ft</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LF29H8330S</t>
+          <t>26ft Box Truck</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>NJ-DC1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
+        <v>312.01</v>
+      </c>
+      <c r="D2" t="n">
+        <v>95.98</v>
+      </c>
+      <c r="E2" t="n">
+        <v>101.97</v>
+      </c>
+      <c r="F2" t="n">
+        <v>9921</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1767.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L001</t>
+          <t>53ft</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>WM4000HWA</t>
+          <t>53ft Dry Van Trailer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NJ-DC1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>L001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>DLEX4000W</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NJ-DC1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>L001</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>LDFN4542S</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>NJ-DC1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>L001</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>LMV1764ST</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>NJ-DC1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>L002</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>OLED65C4PUA</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>40</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CA-DC3</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>L002</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>OLED77C4PUA</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>20</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>CA-DC3</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>L002</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>OLED55C4PUA</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>30</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>CA-DC3</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>L002</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>75QNED85TUA</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>15</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>CA-DC3</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>L003</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>LF25S6560S</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>10</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>TX-DC2</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>L003</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>OLED65C4PUA</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>20</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>TX-DC2</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>L003</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>27GR93U-B</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>50</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TX-DC2</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>L003</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>32GP850-B</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>40</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TX-DC2</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>L003</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>LMC0975ST</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>30</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>TX-DC2</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>53ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>L004</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>OLED55C4PUA</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>15</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>FL-DC4</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>L004</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>OLED65C4PUA</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>12</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>FL-DC4</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>L004</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>32GX850A-B</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>20</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>FL-DC4</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>26ft</t>
-        </is>
+        <v>635.98</v>
+      </c>
+      <c r="D3" t="n">
+        <v>102.01</v>
+      </c>
+      <c r="E3" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>44092</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3990.9</v>
       </c>
     </row>
   </sheetData>
@@ -2279,98 +1840,549 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>load_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>model_code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>destination</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>pickup_date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>truck_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>display_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>length_mm</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>width_mm</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>height_mm</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>max_payload_kg</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>cargo_volume_cbm</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LF29H8330S</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NJ-DC1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>26ft</t>
         </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>26ft Box Truck</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>7925</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2438</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2590</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4500</v>
-      </c>
-      <c r="G2" t="n">
-        <v>50.04</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WM4000HWA</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NJ-DC1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DLEX4000W</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NJ-DC1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LDFN4542S</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NJ-DC1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LMV1764ST</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NJ-DC1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OLED65C4PUA</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CA-DC3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>53ft</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>53ft Dry Van Trailer</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>16154</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2591</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2700</v>
-      </c>
-      <c r="F3" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>113.01</v>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>OLED77C4PUA</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CA-DC3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>OLED55C4PUA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CA-DC3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>75QNED85TUA</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CA-DC3</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LF25S6560S</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TX-DC2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>OLED65C4PUA</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TX-DC2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>27GR93U-B</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TX-DC2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>32GP850-B</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>40</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TX-DC2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LMC0975ST</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TX-DC2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>53ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>L004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>OLED55C4PUA</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FL-DC4</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>L004</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>OLED65C4PUA</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FL-DC4</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>L004</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>32GX850A-B</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FL-DC4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>26ft</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: update Truck_Master to industry-standard specs
26ft Box Truck (Penske Non-CDL — most common commercial fleet class):
- Interior: 311 x 97 x 97 in (25'11" x 8'1" x 8'1")
- Payload: 10,000 lb
- Cargo: 1,700 ft^3

53ft Dry Van Trailer (Wabash DuraPlate HD industry standard):
- Interior: 629 x 101 x 110 in (52'5" x 8'5" x 9'2")
- Payload: 45,000 lb
- Cargo: 4,054 ft^3

Web-verified against Penske, Hale Trailer, Wabash specs.
Previous values had 53ft height -4 in too low (106.3 vs industry 110)
and 26ft was on the higher-spec side (102 in interior height).
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -1787,19 +1787,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>312.01</v>
+        <v>311</v>
       </c>
       <c r="D2" t="n">
-        <v>95.98</v>
+        <v>97</v>
       </c>
       <c r="E2" t="n">
-        <v>101.97</v>
+        <v>97</v>
       </c>
       <c r="F2" t="n">
-        <v>9921</v>
+        <v>10000</v>
       </c>
       <c r="G2" t="n">
-        <v>1767.1</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="3">
@@ -1814,19 +1814,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>635.98</v>
+        <v>629</v>
       </c>
       <c r="D3" t="n">
-        <v>102.01</v>
+        <v>101</v>
       </c>
       <c r="E3" t="n">
-        <v>106.3</v>
+        <v>110</v>
       </c>
       <c r="F3" t="n">
-        <v>44092</v>
+        <v>45000</v>
       </c>
       <c r="G3" t="n">
-        <v>3990.9</v>
+        <v>4054</v>
       </c>
     </row>
   </sheetData>

</xml_diff>